<commit_message>
Adding new insights on inbound insights
</commit_message>
<xml_diff>
--- a/fault_inbound_insights test upload sheet.xlsx
+++ b/fault_inbound_insights test upload sheet.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="44">
   <si>
     <t>agent_type</t>
   </si>
@@ -156,9 +156,6 @@
   </si>
   <si>
     <t>February</t>
-  </si>
-  <si>
-    <t>JANUARY</t>
   </si>
 </sst>
 </file>
@@ -2576,8 +2573,8 @@
       <c r="D19" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>44</v>
+      <c r="E19" s="1">
+        <v>5</v>
       </c>
       <c r="F19" s="1">
         <v>676</v>

</xml_diff>